<commit_message>
Tighten Canva field char limits and add text overflow template guide
Co-authored-by: amirdashbns <amirdashbns@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
+++ b/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Carousel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -626,22 +626,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stop Describing</t>
+          <t>Stop</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Describing</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Your Voice</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>to the AI</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Show It Instead</t>
+          <t>to AI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -651,13 +651,13 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>You've been adding adjectives to your ChatGPT prompts like seasoning a bad meal.</t>
+          <t>You've been adjective-loading your ChatGPT prompts.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>You keep rewriting prompts and still sound generic</t>
+          <t>You still sound generic after months of tweaking</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -667,13 +667,13 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Not by explanation. You can describe your tone for 500 words. It won't stick.</t>
+          <t>Not by explanation. Describe your tone all day.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>You have told ChatGPT to write casual witty and friendly a hundred times</t>
+          <t>You told ChatGPT to sound casual a hundred times</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -683,33 +683,33 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Paste something YOU actually wrote. An email. A post. A newsletter.</t>
+          <t>Paste something YOU actually wrote first.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Then ask it to write the new thing in that style. That is it. Context beats instructions.</t>
+          <t>Then ask for the new thing in that style.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>You have old emails or posts you are proud of sitting in a folder</t>
+          <t>You have old posts sitting in a folder</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Why prompt packs fail you</t>
+          <t>Why prompt packs fail</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>They teach you clever tricks. Not YOUR voice. Everyone using the same prompts sounds the same.</t>
+          <t>They teach tricks. Not YOUR voice.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>You have bought prompt packs and felt nothing changed</t>
+          <t>You bought packs and nothing changed</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -719,17 +719,17 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Build a voice sample library. Feed the AI your real writing before every task.</t>
+          <t>Feed the AI your real writing before every task.</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Instructions set the task. Examples set the voice.</t>
+          <t>Examples set the voice. Instructions set the task.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>You want AI content that passes the would-I-actually-say-this test</t>
+          <t>You want copy that passes the sounds-like-me test</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr"/>
@@ -757,7 +757,7 @@
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>YOUR REAL WRITING.</t>
+          <t>YOUR WRITING.</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">

</xml_diff>

<commit_message>
Reframe Canva integration: words over design, template serves copy
- Philosophy: carousel copy is source of truth; Canva table maps not trims
- Soft char refs for stock template; word-first template redesign guide
- Skill: split across fields/slides instead of shortening for text boxes
- Restore fuller sample CSV

Co-authored-by: amirdashbns <amirdashbns@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
+++ b/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
@@ -626,22 +626,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stop</t>
+          <t>Stop Describing</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Describing</t>
+          <t>Your Voice</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Your Voice</t>
+          <t>to the AI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>to AI</t>
+          <t>Show It Instead</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -651,13 +651,13 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>You've been adjective-loading your ChatGPT prompts.</t>
+          <t>You've been adding adjectives to your ChatGPT prompts like seasoning a bad meal.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>You still sound generic after months of tweaking</t>
+          <t>You keep rewriting prompts and still sound generic</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -667,13 +667,13 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Not by explanation. Describe your tone all day.</t>
+          <t>Not by explanation. You can describe your tone for 500 words. It won't stick.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>You told ChatGPT to sound casual a hundred times</t>
+          <t>You've told ChatGPT to write casual witty and friendly a hundred times</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -683,33 +683,33 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Paste something YOU actually wrote first.</t>
+          <t>Paste something YOU actually wrote. An email. A post. A newsletter.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Then ask for the new thing in that style.</t>
+          <t>Then ask it to write the new thing in that style. That's it. Context beats instructions.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>You have old posts sitting in a folder</t>
+          <t>You have old emails or posts you're proud of sitting in a folder</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Why prompt packs fail</t>
+          <t>Why prompt packs fail you</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>They teach tricks. Not YOUR voice.</t>
+          <t>They teach you clever tricks. Not YOUR voice. Everyone using the same prompts sounds the same.</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>You bought packs and nothing changed</t>
+          <t>You've bought prompt packs and felt nothing changed</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -719,17 +719,17 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Feed the AI your real writing before every task.</t>
+          <t>Build a voice sample library. Feed the AI your real writing before every task.</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Examples set the voice. Instructions set the task.</t>
+          <t>Instructions set the task. Examples set the voice.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>You want copy that passes the sounds-like-me test</t>
+          <t>You want AI content that passes the would-I-actually-say-this test</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr"/>
@@ -757,7 +757,7 @@
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>YOUR WRITING.</t>
+          <t>YOUR REAL WRITING.</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">

</xml_diff>

<commit_message>
Simplify Canva field map: 32 fields, merge title/takeaway/CTA boxes
- Title, Takeaway, CTA_Steps are single fields (no per-line/accent splits)
- Body keeps Heading + P1 + P2 + PerfectIf only
- Pink accents static in template; less overlap and reconnect work
- Update sample CSV/XLSX and skill Phase 8

Co-authored-by: amirdashbns <amirdashbns@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
+++ b/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
@@ -413,376 +413,288 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Title_Line1</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Title_Highlight</t>
+          <t>Body1_Heading</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Title_Line2</t>
+          <t>Body1_P1</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Title_Line3</t>
+          <t>Body1_P2</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Body1_Heading</t>
+          <t>Body1_PerfectIf</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Body1_P1</t>
+          <t>Body2_Heading</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Body1_P2</t>
+          <t>Body2_P1</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Body1_PerfectIf</t>
+          <t>Body2_P2</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Body2_Heading</t>
+          <t>Body2_PerfectIf</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Body2_P1</t>
+          <t>Body3_Heading</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Body2_P2</t>
+          <t>Body3_P1</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Body2_PerfectIf</t>
+          <t>Body3_P2</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Body3_Heading</t>
+          <t>Body3_PerfectIf</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Body3_P1</t>
+          <t>Body4_Heading</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Body3_P2</t>
+          <t>Body4_P1</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Body3_PerfectIf</t>
+          <t>Body4_P2</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>Body4_Heading</t>
+          <t>Body4_PerfectIf</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>Body4_P1</t>
+          <t>Body5_Heading</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>Body4_P2</t>
+          <t>Body5_P1</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>Body4_PerfectIf</t>
+          <t>Body5_P2</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Body5_Heading</t>
+          <t>Body5_PerfectIf</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Body5_P1</t>
+          <t>Body6_Heading</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Body5_P2</t>
+          <t>Body6_P1</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Body5_PerfectIf</t>
+          <t>Body6_P2</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>Body6_Heading</t>
+          <t>Body6_PerfectIf</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Body6_P1</t>
+          <t>Body7_Heading</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>Body6_P2</t>
+          <t>Body7_P1</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>Body6_PerfectIf</t>
+          <t>Body7_P2</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>Body7_Heading</t>
+          <t>Body7_PerfectIf</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
         <is>
-          <t>Body7_P1</t>
+          <t>Takeaway</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>Body7_P2</t>
+          <t>CTA_Question</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr">
         <is>
-          <t>Body7_PerfectIf</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>Takeaway_L1</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Takeaway_Accent</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Takeaway_L2</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>Takeaway_L3</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>CTA_Question</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>CTA_Step1</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>CTA_Step2_Prefix</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>CTA_Keyword</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>CTA_Step2_Suffix</t>
+          <t>CTA_Steps</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stop Describing</t>
+          <t>Stop Describing Your Voice to the AI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Your Voice</t>
+          <t>Here's the deal:</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>to the AI</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Show It Instead</t>
-        </is>
-      </c>
+          <t>You've been adding adjectives to your ChatGPT prompts like seasoning a bad meal.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Here's the deal:</t>
+          <t>You keep rewriting prompts and still sound generic</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>You've been adding adjectives to your ChatGPT prompts like seasoning a bad meal.</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>You keep rewriting prompts and still sound generic</t>
-        </is>
-      </c>
+          <t>AI learns by example</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Not by explanation. You can describe your tone for 500 words. It won't stick.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>AI learns by example</t>
+          <t>You've told ChatGPT to write casual witty and friendly a hundred times</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Not by explanation. You can describe your tone for 500 words. It won't stick.</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
+          <t>The mimic prompt fix</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Paste something YOU actually wrote. An email. A post. A newsletter.</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>You've told ChatGPT to write casual witty and friendly a hundred times</t>
+          <t>Then ask it to write the new thing in that style. That's it. Context beats instructions.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The mimic prompt fix</t>
+          <t>You have old emails or posts you're proud of sitting in a folder</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Paste something YOU actually wrote. An email. A post. A newsletter.</t>
+          <t>Why prompt packs fail you</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Then ask it to write the new thing in that style. That's it. Context beats instructions.</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>You have old emails or posts you're proud of sitting in a folder</t>
-        </is>
-      </c>
+          <t>They teach you clever tricks. Not YOUR voice. Everyone using the same prompts sounds the same.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Why prompt packs fail you</t>
+          <t>You've bought prompt packs and felt nothing changed</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>They teach you clever tricks. Not YOUR voice. Everyone using the same prompts sounds the same.</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr"/>
+          <t>What to do instead</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Build a voice sample library. Feed the AI your real writing before every task.</t>
+        </is>
+      </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>You've bought prompt packs and felt nothing changed</t>
+          <t>Instructions set the task. Examples set the voice.</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>What to do instead</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Build a voice sample library. Feed the AI your real writing before every task.</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Instructions set the task. Examples set the voice.</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
           <t>You want AI content that passes the would-I-actually-say-this test</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>STOP COLLECTING</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>PROMPTS.</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>START FEEDING IT</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>YOUR REAL WRITING.</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>STOP COLLECTING PROMPTS.
+START FEEDING IT YOUR REAL WRITING.</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Found this helpful?</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>1) SAVE FOR LATER</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>2) COMMENT '</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>VOICE</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>' TO GET MY FREE AI VOICE GUIDE</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>1) SAVE FOR LATER
+2) COMMENT 'VOICE' TO GET MY FREE AI VOICE GUIDE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Bulk Create P2 fields: Canva drops empty columns
- Document that empty P2 cells cause Canva to omit those fields entirely
- Fill all P2 cells in sample CSV/XLSX files
- Add sample-canva-strategy-test files with full 7-step data for template testing

Co-authored-by: amirdashbns <amirdashbns@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
+++ b/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
@@ -594,7 +594,11 @@
           <t>You've been adding adjectives to your ChatGPT prompts like seasoning a bad meal.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>More instructions will not fix it. You need a different approach entirely.</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>You keep rewriting prompts and still sound generic</t>
@@ -610,7 +614,11 @@
           <t>Not by explanation. You can describe your tone for 500 words. It won't stick.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>It learns patterns from what you show it — not from what you tell it.</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>You've told ChatGPT to write casual witty and friendly a hundred times</t>
@@ -646,7 +654,11 @@
           <t>They teach you clever tricks. Not YOUR voice. Everyone using the same prompts sounds the same.</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>The prompt-pack industry sold you shortcuts. You needed a system.</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>You've bought prompt packs and felt nothing changed</t>
@@ -672,14 +684,46 @@
           <t>You want AI content that passes the would-I-actually-say-this test</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="AD2" t="inlineStr">
         <is>
           <t>STOP COLLECTING PROMPTS.

</xml_diff>

<commit_message>
Remove PerfectIf fields (25-col schema) + Google Sheets repeat workflow
- Drop Body{N}_PerfectIf from field map and sample CSV/XLSX files
- Add carousel-data-headers-only.csv for Google Sheet setup
- Document faster repeat workflow via persistent Google Sheet data source

Co-authored-by: amirdashbns <amirdashbns@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
+++ b/knowledge/frameworks/instagram-content/sample-canva-bulk-create.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,140 +439,105 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Body1_PerfectIf</t>
+          <t>Body2_Heading</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Body2_Heading</t>
+          <t>Body2_P1</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Body2_P1</t>
+          <t>Body2_P2</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Body2_P2</t>
+          <t>Body3_Heading</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Body2_PerfectIf</t>
+          <t>Body3_P1</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Body3_Heading</t>
+          <t>Body3_P2</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Body3_P1</t>
+          <t>Body4_Heading</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Body3_P2</t>
+          <t>Body4_P1</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Body3_PerfectIf</t>
+          <t>Body4_P2</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Body4_Heading</t>
+          <t>Body5_Heading</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Body4_P1</t>
+          <t>Body5_P1</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Body4_P2</t>
+          <t>Body5_P2</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>Body4_PerfectIf</t>
+          <t>Body6_Heading</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>Body5_Heading</t>
+          <t>Body6_P1</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>Body5_P1</t>
+          <t>Body6_P2</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>Body5_P2</t>
+          <t>Body7_Heading</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Body5_PerfectIf</t>
+          <t>Body7_P1</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Body6_Heading</t>
+          <t>Body7_P2</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Body6_P1</t>
+          <t>Takeaway</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Body6_P2</t>
+          <t>CTA_Question</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
-        <is>
-          <t>Body6_PerfectIf</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Body7_Heading</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Body7_P1</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Body7_P2</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Body7_PerfectIf</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Takeaway</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>CTA_Question</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
         <is>
           <t>CTA_Steps</t>
         </is>
@@ -601,141 +566,106 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>You keep rewriting prompts and still sound generic</t>
+          <t>AI learns by example</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AI learns by example</t>
+          <t>Not by explanation. You can describe your tone for 500 words. It won't stick.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Not by explanation. You can describe your tone for 500 words. It won't stick.</t>
+          <t>It learns patterns from what you show it — not from what you tell it.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>It learns patterns from what you show it — not from what you tell it.</t>
+          <t>The mimic prompt fix</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>You've told ChatGPT to write casual witty and friendly a hundred times</t>
+          <t>Paste something YOU actually wrote. An email. A post. A newsletter.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>The mimic prompt fix</t>
+          <t>Then ask it to write the new thing in that style. That's it. Context beats instructions.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Paste something YOU actually wrote. An email. A post. A newsletter.</t>
+          <t>Why prompt packs fail you</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Then ask it to write the new thing in that style. That's it. Context beats instructions.</t>
+          <t>They teach you clever tricks. Not YOUR voice. Everyone using the same prompts sounds the same.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>You have old emails or posts you're proud of sitting in a folder</t>
+          <t>The prompt-pack industry sold you shortcuts. You needed a system.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Why prompt packs fail you</t>
+          <t>What to do instead</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>They teach you clever tricks. Not YOUR voice. Everyone using the same prompts sounds the same.</t>
+          <t>Build a voice sample library. Feed the AI your real writing before every task.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>The prompt-pack industry sold you shortcuts. You needed a system.</t>
+          <t>Instructions set the task. Examples set the voice.</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>You've bought prompt packs and felt nothing changed</t>
+          <t> </t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>What to do instead</t>
+          <t> </t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Build a voice sample library. Feed the AI your real writing before every task.</t>
+          <t> </t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Instructions set the task. Examples set the voice.</t>
+          <t> </t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>You want AI content that passes the would-I-actually-say-this test</t>
+          <t> </t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t> </t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
         <is>
           <t>STOP COLLECTING PROMPTS.
 START FEEDING IT YOUR REAL WRITING.</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>Found this helpful?</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>1) SAVE FOR LATER
 2) COMMENT 'VOICE' TO GET MY FREE AI VOICE GUIDE</t>

</xml_diff>